<commit_message>
docs: 甘特图更新至 v1.1（Sprint 1 进度 + kv_store 存储层）
参考 软件项目开发计划.md v1.1 / 项目开发时间轴.md v1.1 更新：

- 项目甘特图 sheet：
  - 新增「状态」列：P0 七项任务全部 ✅ 完成（含 kv_store 存储层 PR #5、
    题目只读 API、前端三页）；P1-1 题库写接口 / P1-6 前端对话页 🔶 部分完成
  - 任务表对齐现状：P0-3 更名「数据库层 (users表 + kv_store存储层)」、
    新增 P0-4 题目只读 API、P0-6 更名前端三页、P1-1 拆分为写接口、
    P1-5 更名前端试卷管理页、P1-8 更名测试体系完善 (run_tests.sh四组)
  - 甘特条按状态着色：绿=已完成 / 橙=进行中 / 阶段色=计划
  - 当前周 W2 10/12 列头橙色 ▼ 标注；底部新增图例行（含 kv_store 说明）
  - 标题标注 v1.1 更新于 2026-10-13
- 里程碑 sheet：M1 ✅ 已达成；M2 🔶 进行中（对齐开发计划 v1.1）
- 团队分工 sheet：李俊熠/卢恒毅/戴儒骋行纳入 kv_store、测试体系、
  接口文档整合现状

Co-authored-by: AiWork <noreply@aiwork.local>
</commit_message>
<xml_diff>
--- a/docs/项目开发计划甘特图.xlsx
+++ b/docs/项目开发计划甘特图.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,13 @@
       <name val="Microsoft YaHei"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -57,12 +62,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00ED7D31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ED7D31"/>
+        <fgColor rgb="0022C55E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F59E0B"/>
       </patternFill>
     </fill>
     <fill>
@@ -97,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -105,30 +120,40 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -499,27 +524,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI+题库智能教学平台 - 项目开发计划甘特图 (2026.10-11)</t>
+          <t>AI+题库智能教学平台 - 项目开发计划甘特图 (2026.10-11)｜v1.1 更新于 2026-10-13</t>
         </is>
       </c>
     </row>
@@ -556,851 +582,1013 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>W1 10/05</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>W2 10/12</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>W2 10/12 ▼</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>W3 10/19</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>W4 10/26</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>W5 11/02</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>W6 11/09</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P0 - 核心版本 (第1-2周)</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="5" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>P0-1</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>环境搭建 + CI 配置</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>卢恒毅</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8" t="n"/>
-      <c r="K4" s="8" t="n"/>
-      <c r="L4" s="8" t="n"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>✅ 完成</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="10" t="n"/>
+      <c r="J4" s="10" t="n"/>
+      <c r="K4" s="10" t="n"/>
+      <c r="L4" s="10" t="n"/>
+      <c r="M4" s="10" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>P0-2</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>用户认证系统 (登录/登出/Token/me)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>牛宇歌</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>✅ 完成 (4组回归)</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="10" t="n"/>
+      <c r="L5" s="10" t="n"/>
+      <c r="M5" s="10" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>P0-3</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>数据库表结构设计</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>数据库层 (users表 + kv_store存储层)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>李俊熠</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>✅ 完成 (PR #5)</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="10" t="n"/>
+      <c r="L6" s="10" t="n"/>
+      <c r="M6" s="10" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>P0-4</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>题目只读 API (列表/详情 + 5题seed)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>李俊熠</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>✅ 完成</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="10" t="n"/>
+      <c r="M7" s="10" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>P0-5</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>HTTP 服务框架 (libmicrohttpd)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>卢恒毅</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>✅ 完成</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="10" t="n"/>
+      <c r="K8" s="10" t="n"/>
+      <c r="L8" s="10" t="n"/>
+      <c r="M8" s="10" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>P0-5</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>前端骨架页面</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>P0-6</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>前端骨架页面 (登录/列表/对话三页)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>曹渲东、王英杰</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="n"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>✅ 完成</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="10" t="n"/>
+      <c r="K9" s="10" t="n"/>
+      <c r="L9" s="10" t="n"/>
+      <c r="M9" s="10" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>P0-6</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>项目文档初始化</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>P0-7</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>项目文档初始化 (含 kvstore.md)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>戴儒骋</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="8" t="n"/>
-      <c r="L9" s="8" t="n"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>P1 - 功能版本 (第3-4周)</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>✅ 完成</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="9" t="n"/>
       <c r="J10" s="10" t="n"/>
       <c r="K10" s="10" t="n"/>
       <c r="L10" s="10" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="M10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>P1 - 功能版本 (第3-4周)</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="12" t="n"/>
+      <c r="M11" s="12" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>P1-1</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>题库 CRUD 接口</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>题库写接口 (创建/编辑/归档)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>李俊熠</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="8" t="n"/>
-      <c r="L11" s="8" t="n"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>🔶 只读已上线</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="10" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="10" t="n"/>
+      <c r="M12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>P1-2</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>试卷管理接口</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>李俊熠</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="8" t="n"/>
-      <c r="L12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="n"/>
+      <c r="I13" s="10" t="n"/>
+      <c r="J13" s="14" t="n"/>
+      <c r="K13" s="14" t="n"/>
+      <c r="L13" s="10" t="n"/>
+      <c r="M13" s="10" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>P1-3</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>AI 代理调用实现</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>AI 代理调用实现 (/api/v1/chat)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>刘英哲</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="8" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="8" t="n"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="n"/>
+      <c r="I14" s="10" t="n"/>
+      <c r="J14" s="14" t="n"/>
+      <c r="K14" s="14" t="n"/>
+      <c r="L14" s="10" t="n"/>
+      <c r="M14" s="10" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>P1-4</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>分支对话树</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>刘英哲</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F15" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="8" t="n"/>
-      <c r="I14" s="8" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
-      <c r="L14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="n"/>
+      <c r="I15" s="10" t="n"/>
+      <c r="J15" s="10" t="n"/>
+      <c r="K15" s="14" t="n"/>
+      <c r="L15" s="14" t="n"/>
+      <c r="M15" s="10" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>P1-5</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>前端题库页面</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>前端试卷管理页</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>曹渲东、王英杰</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F16" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="8" t="n"/>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="8" t="n"/>
-      <c r="L15" s="8" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="n"/>
+      <c r="I16" s="10" t="n"/>
+      <c r="J16" s="14" t="n"/>
+      <c r="K16" s="14" t="n"/>
+      <c r="L16" s="10" t="n"/>
+      <c r="M16" s="10" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>P1-6</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>前端 AI 对话页</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>曹渲东、王英杰</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="8" t="n"/>
-      <c r="I16" s="8" t="n"/>
-      <c r="J16" s="11" t="n"/>
-      <c r="K16" s="11" t="n"/>
-      <c r="L16" s="8" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>🔶 页面已上线,待接AI</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="n"/>
+      <c r="I17" s="10" t="n"/>
+      <c r="J17" s="10" t="n"/>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="13" t="n"/>
+      <c r="M17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>P1-7</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>管理后台</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>曹渲东、王英杰</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="8" t="n"/>
-      <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8" t="n"/>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="11" t="n"/>
-      <c r="L17" s="8" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="10" t="n"/>
+      <c r="J18" s="10" t="n"/>
+      <c r="K18" s="14" t="n"/>
+      <c r="L18" s="14" t="n"/>
+      <c r="M18" s="10" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>P1-8</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>冒烟测试完善</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>测试体系完善 (run_tests.sh四组)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>卢恒毅</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="8" t="n"/>
-      <c r="H18" s="8" t="n"/>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="11" t="n"/>
-      <c r="K18" s="8" t="n"/>
-      <c r="L18" s="8" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="14" t="n"/>
+      <c r="K19" s="14" t="n"/>
+      <c r="L19" s="10" t="n"/>
+      <c r="M19" s="10" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>P2 - 增强版本 (第5-6周)</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="13" t="n"/>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="13" t="n"/>
-      <c r="J19" s="13" t="n"/>
-      <c r="K19" s="13" t="n"/>
-      <c r="L19" s="13" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="16" t="n"/>
+      <c r="M20" s="16" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>P2-1</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>重复问题检测</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>刘英哲</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="8" t="n"/>
-      <c r="H20" s="8" t="n"/>
-      <c r="I20" s="8" t="n"/>
-      <c r="J20" s="8" t="n"/>
-      <c r="K20" s="14" t="n"/>
-      <c r="L20" s="14" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="n"/>
+      <c r="I21" s="10" t="n"/>
+      <c r="J21" s="10" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="17" t="n"/>
+      <c r="M21" s="17" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>P2-2</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>内容审核</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>牛宇歌</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F22" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="8" t="n"/>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8" t="n"/>
-      <c r="K21" s="14" t="n"/>
-      <c r="L21" s="8" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="10" t="n"/>
+      <c r="J22" s="10" t="n"/>
+      <c r="K22" s="10" t="n"/>
+      <c r="L22" s="17" t="n"/>
+      <c r="M22" s="10" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>P2-3</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>额度管理系统</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>李俊熠</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F23" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="8" t="n"/>
-      <c r="H22" s="8" t="n"/>
-      <c r="I22" s="8" t="n"/>
-      <c r="J22" s="8" t="n"/>
-      <c r="K22" s="14" t="n"/>
-      <c r="L22" s="14" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="n"/>
+      <c r="I23" s="10" t="n"/>
+      <c r="J23" s="10" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="17" t="n"/>
+      <c r="M23" s="17" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>P2-4</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>通知中心</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>牛宇歌</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F24" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
-      <c r="I23" s="8" t="n"/>
-      <c r="J23" s="8" t="n"/>
-      <c r="K23" s="14" t="n"/>
-      <c r="L23" s="14" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="n"/>
+      <c r="I24" s="10" t="n"/>
+      <c r="J24" s="10" t="n"/>
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="17" t="n"/>
+      <c r="M24" s="17" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>P2-5</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>API 捐赠功能</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>李俊熠</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F25" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="8" t="n"/>
-      <c r="H24" s="8" t="n"/>
-      <c r="I24" s="8" t="n"/>
-      <c r="J24" s="8" t="n"/>
-      <c r="K24" s="8" t="n"/>
-      <c r="L24" s="14" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="n"/>
+      <c r="I25" s="10" t="n"/>
+      <c r="J25" s="10" t="n"/>
+      <c r="K25" s="10" t="n"/>
+      <c r="L25" s="10" t="n"/>
+      <c r="M25" s="17" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>P2-6</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>系统部署 (systemd)</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>卢恒毅</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F26" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="n"/>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="8" t="n"/>
-      <c r="K25" s="14" t="n"/>
-      <c r="L25" s="14" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
+      <c r="J26" s="10" t="n"/>
+      <c r="K26" s="10" t="n"/>
+      <c r="L26" s="17" t="n"/>
+      <c r="M26" s="17" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>P2-7</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>集成测试 + D7 演示</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>全员</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F27" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="8" t="n"/>
-      <c r="H26" s="8" t="n"/>
-      <c r="I26" s="8" t="n"/>
-      <c r="J26" s="8" t="n"/>
-      <c r="K26" s="8" t="n"/>
-      <c r="L26" s="14" t="n"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="10" t="n"/>
+      <c r="J27" s="10" t="n"/>
+      <c r="K27" s="10" t="n"/>
+      <c r="L27" s="10" t="n"/>
+      <c r="M27" s="17" t="n"/>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>图例：✅ 已完成(绿条)　🔶 进行中(橙条)　⬜ 计划(阶段色)　▼ 当前周(W2 10/12)｜kv_store 目录式存储层已合入 main (PR #5)，接口文档 docs/kvstore.md，18 断言单元测试纳入 CI</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A19:C19"/>
+  <mergeCells count="5">
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:M1"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A29:M29"/>
+    <mergeCell ref="A20:C20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1418,145 +1606,145 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>项目里程碑</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>验收标准</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>M1 - 基础框架就绪</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>W1末 (10/11)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>CI跑通 + 登录/登出可用</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
-        <is>
-          <t>进行中</t>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>✅ 已达成</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>M2 - 核心功能完成</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>W2末 (10/18)</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>题库CRUD + AI解答 + 前端可用</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
-        <is>
-          <t>待开始</t>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>🔶 进行中</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>M3 - 功能完善</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>W4末 (11/01)</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>对话树 + 管理后台走通</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
-        <is>
-          <t>待开始</t>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>M4 - 集成测试</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>W5末 (11/08)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>全链路冒烟测试通过</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>待开始</t>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>全链路测试通过</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>M5 - 最终演示</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>W6末 (11/15)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>D7 演示日通过</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>待开始</t>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>⬜ 待开始</t>
         </is>
       </c>
     </row>
@@ -1579,188 +1767,188 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>团队分工表</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>姓名</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>角色</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>负责模块</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>关键产出</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>戴儒骋</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>项目经理/文档</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
-        <is>
-          <t>AGENT.md、api.md、项目计划</t>
-        </is>
-      </c>
-      <c r="D4" s="17" t="inlineStr">
-        <is>
-          <t>全部计划文档 + 接口规范</t>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>AGENT.md、模块接口文档(auth/questions/kvstore)、项目计划</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>全部计划文档 + api.md 整合中</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>卢恒毅</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>技术负责人/安全</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>CI/CD、架构审查、冒烟测试</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="inlineStr">
-        <is>
-          <t>CI流水线 + 全链路测试</t>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>CI/CD、架构审查、测试体系(run_tests.sh)</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>CI流水线 + 四组自动化测试</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>牛宇歌</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>后端-认证</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>auth.c/h, 登录/注册/鉴权</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
-        <is>
-          <t>认证系统 + 通知中心</t>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>认证系统(4组回归) + 通知中心</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>李俊熠</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>后端-题库</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>题库CRUD、db.c扩展</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>题库API + 额度管理</t>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>题库CRUD、kv_store存储层、db.c扩展</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>题目只读API + kv_store存储层(PR #5)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>刘英哲</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>后端-AI</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>ai_client.c/h, 对话树</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>AI代理 + 去重检测</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>曹渲东</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>前端</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>web/ 题库+管理后台页</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>前端页面开发</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>王英杰</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>前端</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>web/ AI对话+个人中心页</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>前端页面开发</t>
         </is>

</xml_diff>